<commit_message>
"Updated the graph feature code to resolve null issues"
</commit_message>
<xml_diff>
--- a/outputs/EDA_transaction_with_graph_features.xlsx
+++ b/outputs/EDA_transaction_with_graph_features.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="9" documentId="11_E24FADE411B2256218ECC4A2B92D12481F1AF638" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{364325F6-088C-40C4-B1CF-05FEE11C433A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_Overview" sheetId="1" r:id="rId1"/>
@@ -3497,10 +3497,6 @@
     <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3555,6 +3551,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3570,6 +3570,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -23448,7 +23452,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="43" t="s">
         <v>69</v>
       </c>
     </row>
@@ -48510,15 +48514,15 @@
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22" style="48" customWidth="1"/>
-    <col min="2" max="2" width="35" style="48" customWidth="1"/>
-    <col min="3" max="3" width="60" style="48" customWidth="1"/>
+    <col min="1" max="1" width="22" style="46" customWidth="1"/>
+    <col min="2" max="2" width="35" style="46" customWidth="1"/>
+    <col min="3" max="3" width="60" style="46" customWidth="1"/>
     <col min="4" max="4" width="70" customWidth="1"/>
     <col min="5" max="5" width="35" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="44" t="s">
         <v>487</v>
       </c>
     </row>
@@ -48540,10 +48544,10 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="47" t="s">
         <v>492</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="47" t="s">
         <v>493</v>
       </c>
       <c r="C3" s="38" t="s">
@@ -48557,10 +48561,10 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="47" t="s">
         <v>492</v>
       </c>
-      <c r="B4" s="49" t="s">
+      <c r="B4" s="47" t="s">
         <v>497</v>
       </c>
       <c r="C4" s="38" t="s">
@@ -48574,13 +48578,13 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="50" t="s">
+      <c r="A5" s="48" t="s">
         <v>178</v>
       </c>
-      <c r="B5" s="50" t="s">
+      <c r="B5" s="48" t="s">
         <v>181</v>
       </c>
-      <c r="C5" s="56" t="s">
+      <c r="C5" s="54" t="s">
         <v>501</v>
       </c>
       <c r="D5" s="26" t="s">
@@ -48591,13 +48595,13 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="48" t="s">
         <v>178</v>
       </c>
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="48" t="s">
         <v>177</v>
       </c>
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="54" t="s">
         <v>504</v>
       </c>
       <c r="D6" s="26" t="s">
@@ -48608,13 +48612,13 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="50" t="s">
+      <c r="A7" s="48" t="s">
         <v>178</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="48" t="s">
         <v>184</v>
       </c>
-      <c r="C7" s="56" t="s">
+      <c r="C7" s="54" t="s">
         <v>507</v>
       </c>
       <c r="D7" s="26" t="s">
@@ -48625,13 +48629,13 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="51" t="s">
+      <c r="A8" s="49" t="s">
         <v>167</v>
       </c>
-      <c r="B8" s="51" t="s">
+      <c r="B8" s="49" t="s">
         <v>510</v>
       </c>
-      <c r="C8" s="57" t="s">
+      <c r="C8" s="55" t="s">
         <v>511</v>
       </c>
       <c r="D8" s="24" t="s">
@@ -48642,13 +48646,13 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="51" t="s">
+      <c r="A9" s="49" t="s">
         <v>167</v>
       </c>
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="49" t="s">
         <v>514</v>
       </c>
-      <c r="C9" s="57" t="s">
+      <c r="C9" s="55" t="s">
         <v>515</v>
       </c>
       <c r="D9" s="24" t="s">
@@ -48659,13 +48663,13 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="51" t="s">
+      <c r="A10" s="49" t="s">
         <v>167</v>
       </c>
-      <c r="B10" s="51" t="s">
+      <c r="B10" s="49" t="s">
         <v>166</v>
       </c>
-      <c r="C10" s="57" t="s">
+      <c r="C10" s="55" t="s">
         <v>518</v>
       </c>
       <c r="D10" s="24" t="s">
@@ -48676,13 +48680,13 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="51" t="s">
+      <c r="A11" s="49" t="s">
         <v>167</v>
       </c>
-      <c r="B11" s="51" t="s">
+      <c r="B11" s="49" t="s">
         <v>521</v>
       </c>
-      <c r="C11" s="57" t="s">
+      <c r="C11" s="55" t="s">
         <v>522</v>
       </c>
       <c r="D11" s="24" t="s">
@@ -48693,13 +48697,13 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="51" t="s">
+      <c r="A12" s="49" t="s">
         <v>525</v>
       </c>
-      <c r="B12" s="51" t="s">
+      <c r="B12" s="49" t="s">
         <v>526</v>
       </c>
-      <c r="C12" s="57" t="s">
+      <c r="C12" s="55" t="s">
         <v>527</v>
       </c>
       <c r="D12" s="24" t="s">
@@ -48710,13 +48714,13 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="52" t="s">
+      <c r="A13" s="50" t="s">
         <v>429</v>
       </c>
-      <c r="B13" s="52" t="s">
+      <c r="B13" s="50" t="s">
         <v>428</v>
       </c>
-      <c r="C13" s="58" t="s">
+      <c r="C13" s="56" t="s">
         <v>530</v>
       </c>
       <c r="D13" s="12" t="s">
@@ -48727,13 +48731,13 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="52" t="s">
+      <c r="A14" s="50" t="s">
         <v>429</v>
       </c>
-      <c r="B14" s="52" t="s">
+      <c r="B14" s="50" t="s">
         <v>435</v>
       </c>
-      <c r="C14" s="58" t="s">
+      <c r="C14" s="56" t="s">
         <v>533</v>
       </c>
       <c r="D14" s="12" t="s">
@@ -48744,13 +48748,13 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="52" t="s">
+      <c r="A15" s="50" t="s">
         <v>429</v>
       </c>
-      <c r="B15" s="52" t="s">
+      <c r="B15" s="50" t="s">
         <v>438</v>
       </c>
-      <c r="C15" s="58" t="s">
+      <c r="C15" s="56" t="s">
         <v>536</v>
       </c>
       <c r="D15" s="12" t="s">
@@ -48761,13 +48765,13 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="52" t="s">
+      <c r="A16" s="50" t="s">
         <v>475</v>
       </c>
-      <c r="B16" s="52" t="s">
+      <c r="B16" s="50" t="s">
         <v>474</v>
       </c>
-      <c r="C16" s="58" t="s">
+      <c r="C16" s="56" t="s">
         <v>538</v>
       </c>
       <c r="D16" s="12" t="s">
@@ -48778,13 +48782,13 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="52" t="s">
+      <c r="A17" s="50" t="s">
         <v>475</v>
       </c>
-      <c r="B17" s="52" t="s">
+      <c r="B17" s="50" t="s">
         <v>484</v>
       </c>
-      <c r="C17" s="58" t="s">
+      <c r="C17" s="56" t="s">
         <v>541</v>
       </c>
       <c r="D17" s="12" t="s">
@@ -48795,10 +48799,10 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="53" t="s">
+      <c r="A18" s="51" t="s">
         <v>452</v>
       </c>
-      <c r="B18" s="53" t="s">
+      <c r="B18" s="51" t="s">
         <v>451</v>
       </c>
       <c r="C18" s="9" t="s">
@@ -48812,10 +48816,10 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="53" t="s">
+      <c r="A19" s="51" t="s">
         <v>452</v>
       </c>
-      <c r="B19" s="53" t="s">
+      <c r="B19" s="51" t="s">
         <v>455</v>
       </c>
       <c r="C19" s="9" t="s">
@@ -48829,10 +48833,10 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="53" t="s">
+      <c r="A20" s="51" t="s">
         <v>452</v>
       </c>
-      <c r="B20" s="53" t="s">
+      <c r="B20" s="51" t="s">
         <v>458</v>
       </c>
       <c r="C20" s="9" t="s">
@@ -48846,13 +48850,13 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="54" t="s">
+      <c r="A21" s="52" t="s">
         <v>442</v>
       </c>
-      <c r="B21" s="54" t="s">
+      <c r="B21" s="52" t="s">
         <v>441</v>
       </c>
-      <c r="C21" s="59" t="s">
+      <c r="C21" s="57" t="s">
         <v>550</v>
       </c>
       <c r="D21" s="18" t="s">
@@ -48863,13 +48867,13 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="54" t="s">
+      <c r="A22" s="52" t="s">
         <v>442</v>
       </c>
-      <c r="B22" s="54" t="s">
+      <c r="B22" s="52" t="s">
         <v>461</v>
       </c>
-      <c r="C22" s="59" t="s">
+      <c r="C22" s="57" t="s">
         <v>552</v>
       </c>
       <c r="D22" s="18" t="s">
@@ -48880,13 +48884,13 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="54" t="s">
+      <c r="A23" s="52" t="s">
         <v>442</v>
       </c>
-      <c r="B23" s="54" t="s">
+      <c r="B23" s="52" t="s">
         <v>464</v>
       </c>
-      <c r="C23" s="59" t="s">
+      <c r="C23" s="57" t="s">
         <v>555</v>
       </c>
       <c r="D23" s="18" t="s">
@@ -48897,13 +48901,13 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="54" t="s">
+      <c r="A24" s="52" t="s">
         <v>442</v>
       </c>
-      <c r="B24" s="54" t="s">
+      <c r="B24" s="52" t="s">
         <v>467</v>
       </c>
-      <c r="C24" s="59" t="s">
+      <c r="C24" s="57" t="s">
         <v>558</v>
       </c>
       <c r="D24" s="18" t="s">
@@ -48914,10 +48918,10 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="55" t="s">
+      <c r="A25" s="53" t="s">
         <v>471</v>
       </c>
-      <c r="B25" s="55" t="s">
+      <c r="B25" s="53" t="s">
         <v>470</v>
       </c>
       <c r="C25" s="31" t="s">
@@ -65034,14 +65038,14 @@
       <c r="F3" s="40"/>
     </row>
     <row r="4" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="61" t="s">
         <v>941</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
+      <c r="B4" s="62"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
@@ -65266,14 +65270,14 @@
       <c r="F24" s="40"/>
     </row>
     <row r="25" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="43" t="s">
+      <c r="A25" s="61" t="s">
         <v>978</v>
       </c>
-      <c r="B25" s="44"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="44"/>
-      <c r="F25" s="44"/>
+      <c r="B25" s="62"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="62"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
@@ -65498,14 +65502,14 @@
       <c r="F45" s="40"/>
     </row>
     <row r="46" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="43" t="s">
+      <c r="A46" s="61" t="s">
         <v>992</v>
       </c>
-      <c r="B46" s="44"/>
-      <c r="C46" s="44"/>
-      <c r="D46" s="44"/>
-      <c r="E46" s="44"/>
-      <c r="F46" s="44"/>
+      <c r="B46" s="62"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="62"/>
+      <c r="E46" s="62"/>
+      <c r="F46" s="62"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
@@ -65730,14 +65734,14 @@
       <c r="F66" s="40"/>
     </row>
     <row r="67" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="43" t="s">
+      <c r="A67" s="61" t="s">
         <v>1005</v>
       </c>
-      <c r="B67" s="44"/>
-      <c r="C67" s="44"/>
-      <c r="D67" s="44"/>
-      <c r="E67" s="44"/>
-      <c r="F67" s="44"/>
+      <c r="B67" s="62"/>
+      <c r="C67" s="62"/>
+      <c r="D67" s="62"/>
+      <c r="E67" s="62"/>
+      <c r="F67" s="62"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="8" t="s">
@@ -65962,14 +65966,14 @@
       <c r="F87" s="40"/>
     </row>
     <row r="88" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="43" t="s">
+      <c r="A88" s="61" t="s">
         <v>1021</v>
       </c>
-      <c r="B88" s="44"/>
-      <c r="C88" s="44"/>
-      <c r="D88" s="44"/>
-      <c r="E88" s="44"/>
-      <c r="F88" s="44"/>
+      <c r="B88" s="62"/>
+      <c r="C88" s="62"/>
+      <c r="D88" s="62"/>
+      <c r="E88" s="62"/>
+      <c r="F88" s="62"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="8" t="s">
@@ -82129,7 +82133,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A36" s="36" t="s">
         <v>484</v>
       </c>
@@ -82320,10 +82324,10 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="2" width="14" style="47" customWidth="1"/>
-    <col min="3" max="3" width="12" style="47" customWidth="1"/>
-    <col min="4" max="4" width="14" style="47" customWidth="1"/>
-    <col min="5" max="5" width="15" style="47" customWidth="1"/>
+    <col min="2" max="2" width="14" style="45" customWidth="1"/>
+    <col min="3" max="3" width="12" style="45" customWidth="1"/>
+    <col min="4" max="4" width="14" style="45" customWidth="1"/>
+    <col min="5" max="5" width="15" style="45" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" x14ac:dyDescent="0.3">
@@ -82335,10 +82339,10 @@
       <c r="A3" s="33" t="s">
         <v>648</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -82361,16 +82365,16 @@
       <c r="A5" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="61">
+      <c r="B5" s="59">
         <v>118797</v>
       </c>
-      <c r="C5" s="61" t="s">
+      <c r="C5" s="59" t="s">
         <v>651</v>
       </c>
-      <c r="D5" s="61">
+      <c r="D5" s="59">
         <v>10132</v>
       </c>
-      <c r="E5" s="61" t="s">
+      <c r="E5" s="59" t="s">
         <v>652</v>
       </c>
     </row>
@@ -82378,16 +82382,16 @@
       <c r="A6" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="62">
+      <c r="B6" s="60">
         <v>75392</v>
       </c>
-      <c r="C6" s="62" t="s">
+      <c r="C6" s="60" t="s">
         <v>653</v>
       </c>
-      <c r="D6" s="62">
+      <c r="D6" s="60">
         <v>10219</v>
       </c>
-      <c r="E6" s="62" t="s">
+      <c r="E6" s="60" t="s">
         <v>654</v>
       </c>
     </row>
@@ -82395,16 +82399,16 @@
       <c r="A7" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B7" s="61">
+      <c r="B7" s="59">
         <v>24143</v>
       </c>
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="59" t="s">
         <v>655</v>
       </c>
-      <c r="D7" s="61">
+      <c r="D7" s="59">
         <v>2672</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="59" t="s">
         <v>656</v>
       </c>
     </row>
@@ -82412,16 +82416,16 @@
       <c r="A8" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B8" s="62">
+      <c r="B8" s="60">
         <v>24120</v>
       </c>
-      <c r="C8" s="62" t="s">
+      <c r="C8" s="60" t="s">
         <v>657</v>
       </c>
-      <c r="D8" s="62">
+      <c r="D8" s="60">
         <v>2499</v>
       </c>
-      <c r="E8" s="62" t="s">
+      <c r="E8" s="60" t="s">
         <v>658</v>
       </c>
     </row>
@@ -82429,10 +82433,10 @@
       <c r="A11" s="33" t="s">
         <v>659</v>
       </c>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
+      <c r="B11" s="58"/>
+      <c r="C11" s="58"/>
+      <c r="D11" s="58"/>
+      <c r="E11" s="58"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
@@ -82455,16 +82459,16 @@
       <c r="A13" s="6" t="s">
         <v>660</v>
       </c>
-      <c r="B13" s="61">
+      <c r="B13" s="59">
         <v>39838</v>
       </c>
-      <c r="C13" s="61" t="s">
+      <c r="C13" s="59" t="s">
         <v>661</v>
       </c>
-      <c r="D13" s="61">
+      <c r="D13" s="59">
         <v>3428</v>
       </c>
-      <c r="E13" s="61" t="s">
+      <c r="E13" s="59" t="s">
         <v>662</v>
       </c>
     </row>
@@ -82472,16 +82476,16 @@
       <c r="A14" s="4" t="s">
         <v>663</v>
       </c>
-      <c r="B14" s="62">
+      <c r="B14" s="60">
         <v>39497</v>
       </c>
-      <c r="C14" s="62" t="s">
+      <c r="C14" s="60" t="s">
         <v>664</v>
       </c>
-      <c r="D14" s="62">
+      <c r="D14" s="60">
         <v>3373</v>
       </c>
-      <c r="E14" s="62" t="s">
+      <c r="E14" s="60" t="s">
         <v>652</v>
       </c>
     </row>
@@ -82489,16 +82493,16 @@
       <c r="A15" s="6" t="s">
         <v>665</v>
       </c>
-      <c r="B15" s="61">
+      <c r="B15" s="59">
         <v>39462</v>
       </c>
-      <c r="C15" s="61" t="s">
+      <c r="C15" s="59" t="s">
         <v>666</v>
       </c>
-      <c r="D15" s="61">
+      <c r="D15" s="59">
         <v>3331</v>
       </c>
-      <c r="E15" s="61" t="s">
+      <c r="E15" s="59" t="s">
         <v>667</v>
       </c>
     </row>
@@ -82506,16 +82510,16 @@
       <c r="A16" s="4" t="s">
         <v>668</v>
       </c>
-      <c r="B16" s="62">
+      <c r="B16" s="60">
         <v>25291</v>
       </c>
-      <c r="C16" s="62" t="s">
+      <c r="C16" s="60" t="s">
         <v>669</v>
       </c>
-      <c r="D16" s="62">
+      <c r="D16" s="60">
         <v>3507</v>
       </c>
-      <c r="E16" s="62" t="s">
+      <c r="E16" s="60" t="s">
         <v>670</v>
       </c>
     </row>
@@ -82523,16 +82527,16 @@
       <c r="A17" s="6" t="s">
         <v>671</v>
       </c>
-      <c r="B17" s="61">
+      <c r="B17" s="59">
         <v>25274</v>
       </c>
-      <c r="C17" s="61" t="s">
+      <c r="C17" s="59" t="s">
         <v>672</v>
       </c>
-      <c r="D17" s="61">
+      <c r="D17" s="59">
         <v>3446</v>
       </c>
-      <c r="E17" s="61" t="s">
+      <c r="E17" s="59" t="s">
         <v>654</v>
       </c>
     </row>
@@ -82540,16 +82544,16 @@
       <c r="A18" s="4" t="s">
         <v>673</v>
       </c>
-      <c r="B18" s="62">
+      <c r="B18" s="60">
         <v>24827</v>
       </c>
-      <c r="C18" s="62" t="s">
+      <c r="C18" s="60" t="s">
         <v>674</v>
       </c>
-      <c r="D18" s="62">
+      <c r="D18" s="60">
         <v>3266</v>
       </c>
-      <c r="E18" s="62" t="s">
+      <c r="E18" s="60" t="s">
         <v>675</v>
       </c>
     </row>
@@ -82557,16 +82561,16 @@
       <c r="A19" s="6" t="s">
         <v>676</v>
       </c>
-      <c r="B19" s="61">
+      <c r="B19" s="59">
         <v>20224</v>
       </c>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="59" t="s">
         <v>677</v>
       </c>
-      <c r="D19" s="61">
+      <c r="D19" s="59">
         <v>2219</v>
       </c>
-      <c r="E19" s="61" t="s">
+      <c r="E19" s="59" t="s">
         <v>678</v>
       </c>
     </row>
@@ -82574,16 +82578,16 @@
       <c r="A20" s="4" t="s">
         <v>679</v>
       </c>
-      <c r="B20" s="62">
+      <c r="B20" s="60">
         <v>12083</v>
       </c>
-      <c r="C20" s="62" t="s">
+      <c r="C20" s="60" t="s">
         <v>680</v>
       </c>
-      <c r="D20" s="62">
+      <c r="D20" s="60">
         <v>1309</v>
       </c>
-      <c r="E20" s="62" t="s">
+      <c r="E20" s="60" t="s">
         <v>681</v>
       </c>
     </row>
@@ -82591,16 +82595,16 @@
       <c r="A21" s="6" t="s">
         <v>682</v>
       </c>
-      <c r="B21" s="61">
+      <c r="B21" s="59">
         <v>8012</v>
       </c>
-      <c r="C21" s="61" t="s">
+      <c r="C21" s="59" t="s">
         <v>683</v>
       </c>
-      <c r="D21" s="61">
+      <c r="D21" s="59">
         <v>870</v>
       </c>
-      <c r="E21" s="61" t="s">
+      <c r="E21" s="59" t="s">
         <v>684</v>
       </c>
     </row>
@@ -82608,16 +82612,16 @@
       <c r="A22" s="4" t="s">
         <v>685</v>
       </c>
-      <c r="B22" s="62">
+      <c r="B22" s="60">
         <v>7944</v>
       </c>
-      <c r="C22" s="62" t="s">
+      <c r="C22" s="60" t="s">
         <v>686</v>
       </c>
-      <c r="D22" s="62">
+      <c r="D22" s="60">
         <v>773</v>
       </c>
-      <c r="E22" s="62" t="s">
+      <c r="E22" s="60" t="s">
         <v>687</v>
       </c>
     </row>
@@ -82625,10 +82629,10 @@
       <c r="A25" s="33" t="s">
         <v>688</v>
       </c>
-      <c r="B25" s="60"/>
-      <c r="C25" s="60"/>
-      <c r="D25" s="60"/>
-      <c r="E25" s="60"/>
+      <c r="B25" s="58"/>
+      <c r="C25" s="58"/>
+      <c r="D25" s="58"/>
+      <c r="E25" s="58"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
@@ -82651,16 +82655,16 @@
       <c r="A27" s="6" t="s">
         <v>689</v>
       </c>
-      <c r="B27" s="61">
+      <c r="B27" s="59">
         <v>123065</v>
       </c>
-      <c r="C27" s="61" t="s">
+      <c r="C27" s="59" t="s">
         <v>690</v>
       </c>
-      <c r="D27" s="61">
+      <c r="D27" s="59">
         <v>12649</v>
       </c>
-      <c r="E27" s="61" t="s">
+      <c r="E27" s="59" t="s">
         <v>691</v>
       </c>
     </row>
@@ -82668,16 +82672,16 @@
       <c r="A28" s="4" t="s">
         <v>692</v>
       </c>
-      <c r="B28" s="62">
+      <c r="B28" s="60">
         <v>74210</v>
       </c>
-      <c r="C28" s="62" t="s">
+      <c r="C28" s="60" t="s">
         <v>693</v>
       </c>
-      <c r="D28" s="62">
+      <c r="D28" s="60">
         <v>8104</v>
       </c>
-      <c r="E28" s="62" t="s">
+      <c r="E28" s="60" t="s">
         <v>684</v>
       </c>
     </row>
@@ -82685,16 +82689,16 @@
       <c r="A29" s="6" t="s">
         <v>694</v>
       </c>
-      <c r="B29" s="61">
+      <c r="B29" s="59">
         <v>45177</v>
       </c>
-      <c r="C29" s="61" t="s">
+      <c r="C29" s="59" t="s">
         <v>695</v>
       </c>
-      <c r="D29" s="61">
+      <c r="D29" s="59">
         <v>4769</v>
       </c>
-      <c r="E29" s="61" t="s">
+      <c r="E29" s="59" t="s">
         <v>696</v>
       </c>
     </row>
@@ -82702,10 +82706,10 @@
       <c r="A32" s="33" t="s">
         <v>697</v>
       </c>
-      <c r="B32" s="60"/>
-      <c r="C32" s="60"/>
-      <c r="D32" s="60"/>
-      <c r="E32" s="60"/>
+      <c r="B32" s="58"/>
+      <c r="C32" s="58"/>
+      <c r="D32" s="58"/>
+      <c r="E32" s="58"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
@@ -82728,16 +82732,16 @@
       <c r="A34" s="4" t="s">
         <v>689</v>
       </c>
-      <c r="B34" s="62">
+      <c r="B34" s="60">
         <v>122388</v>
       </c>
-      <c r="C34" s="62" t="s">
+      <c r="C34" s="60" t="s">
         <v>698</v>
       </c>
-      <c r="D34" s="62">
+      <c r="D34" s="60">
         <v>13060</v>
       </c>
-      <c r="E34" s="62" t="s">
+      <c r="E34" s="60" t="s">
         <v>699</v>
       </c>
     </row>
@@ -82745,16 +82749,16 @@
       <c r="A35" s="6" t="s">
         <v>694</v>
       </c>
-      <c r="B35" s="61">
+      <c r="B35" s="59">
         <v>74256</v>
       </c>
-      <c r="C35" s="61" t="s">
+      <c r="C35" s="59" t="s">
         <v>700</v>
       </c>
-      <c r="D35" s="61">
+      <c r="D35" s="59">
         <v>7644</v>
       </c>
-      <c r="E35" s="61" t="s">
+      <c r="E35" s="59" t="s">
         <v>691</v>
       </c>
     </row>
@@ -82762,16 +82766,16 @@
       <c r="A36" s="4" t="s">
         <v>692</v>
       </c>
-      <c r="B36" s="62">
+      <c r="B36" s="60">
         <v>45808</v>
       </c>
-      <c r="C36" s="62" t="s">
+      <c r="C36" s="60" t="s">
         <v>701</v>
       </c>
-      <c r="D36" s="62">
+      <c r="D36" s="60">
         <v>4818</v>
       </c>
-      <c r="E36" s="62" t="s">
+      <c r="E36" s="60" t="s">
         <v>702</v>
       </c>
     </row>
@@ -82779,10 +82783,10 @@
       <c r="A39" s="33" t="s">
         <v>703</v>
       </c>
-      <c r="B39" s="60"/>
-      <c r="C39" s="60"/>
-      <c r="D39" s="60"/>
-      <c r="E39" s="60"/>
+      <c r="B39" s="58"/>
+      <c r="C39" s="58"/>
+      <c r="D39" s="58"/>
+      <c r="E39" s="58"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
@@ -82805,16 +82809,16 @@
       <c r="A41" s="6" t="s">
         <v>704</v>
       </c>
-      <c r="B41" s="61">
+      <c r="B41" s="59">
         <v>75170</v>
       </c>
-      <c r="C41" s="61" t="s">
+      <c r="C41" s="59" t="s">
         <v>705</v>
       </c>
-      <c r="D41" s="61">
+      <c r="D41" s="59">
         <v>7883</v>
       </c>
-      <c r="E41" s="61" t="s">
+      <c r="E41" s="59" t="s">
         <v>702</v>
       </c>
     </row>
@@ -82822,16 +82826,16 @@
       <c r="A42" s="4" t="s">
         <v>706</v>
       </c>
-      <c r="B42" s="62">
+      <c r="B42" s="60">
         <v>34582</v>
       </c>
-      <c r="C42" s="62" t="s">
+      <c r="C42" s="60" t="s">
         <v>707</v>
       </c>
-      <c r="D42" s="62">
+      <c r="D42" s="60">
         <v>3644</v>
       </c>
-      <c r="E42" s="62" t="s">
+      <c r="E42" s="60" t="s">
         <v>702</v>
       </c>
     </row>
@@ -82839,16 +82843,16 @@
       <c r="A43" s="6" t="s">
         <v>708</v>
       </c>
-      <c r="B43" s="61">
+      <c r="B43" s="59">
         <v>31371</v>
       </c>
-      <c r="C43" s="61" t="s">
+      <c r="C43" s="59" t="s">
         <v>709</v>
       </c>
-      <c r="D43" s="61">
+      <c r="D43" s="59">
         <v>3087</v>
       </c>
-      <c r="E43" s="61" t="s">
+      <c r="E43" s="59" t="s">
         <v>710</v>
       </c>
     </row>
@@ -82856,16 +82860,16 @@
       <c r="A44" s="4" t="s">
         <v>711</v>
       </c>
-      <c r="B44" s="62">
+      <c r="B44" s="60">
         <v>23586</v>
       </c>
-      <c r="C44" s="62" t="s">
+      <c r="C44" s="60" t="s">
         <v>712</v>
       </c>
-      <c r="D44" s="62">
+      <c r="D44" s="60">
         <v>2671</v>
       </c>
-      <c r="E44" s="62" t="s">
+      <c r="E44" s="60" t="s">
         <v>713</v>
       </c>
     </row>
@@ -82873,16 +82877,16 @@
       <c r="A45" s="6" t="s">
         <v>714</v>
       </c>
-      <c r="B45" s="61">
+      <c r="B45" s="59">
         <v>22229</v>
       </c>
-      <c r="C45" s="61" t="s">
+      <c r="C45" s="59" t="s">
         <v>715</v>
       </c>
-      <c r="D45" s="61">
+      <c r="D45" s="59">
         <v>2540</v>
       </c>
-      <c r="E45" s="61" t="s">
+      <c r="E45" s="59" t="s">
         <v>716</v>
       </c>
     </row>
@@ -82890,16 +82894,16 @@
       <c r="A46" s="4" t="s">
         <v>717</v>
       </c>
-      <c r="B46" s="62">
+      <c r="B46" s="60">
         <v>20178</v>
       </c>
-      <c r="C46" s="62" t="s">
+      <c r="C46" s="60" t="s">
         <v>718</v>
       </c>
-      <c r="D46" s="62">
+      <c r="D46" s="60">
         <v>1909</v>
       </c>
-      <c r="E46" s="62" t="s">
+      <c r="E46" s="60" t="s">
         <v>719</v>
       </c>
     </row>
@@ -82907,16 +82911,16 @@
       <c r="A47" s="6" t="s">
         <v>720</v>
       </c>
-      <c r="B47" s="61">
+      <c r="B47" s="59">
         <v>19247</v>
       </c>
-      <c r="C47" s="61" t="s">
+      <c r="C47" s="59" t="s">
         <v>721</v>
       </c>
-      <c r="D47" s="61">
+      <c r="D47" s="59">
         <v>2057</v>
       </c>
-      <c r="E47" s="61" t="s">
+      <c r="E47" s="59" t="s">
         <v>699</v>
       </c>
     </row>
@@ -82924,16 +82928,16 @@
       <c r="A48" s="4" t="s">
         <v>722</v>
       </c>
-      <c r="B48" s="62">
+      <c r="B48" s="60">
         <v>16089</v>
       </c>
-      <c r="C48" s="62" t="s">
+      <c r="C48" s="60" t="s">
         <v>723</v>
       </c>
-      <c r="D48" s="62">
+      <c r="D48" s="60">
         <v>1731</v>
       </c>
-      <c r="E48" s="62" t="s">
+      <c r="E48" s="60" t="s">
         <v>681</v>
       </c>
     </row>
@@ -82941,10 +82945,10 @@
       <c r="A51" s="33" t="s">
         <v>724</v>
       </c>
-      <c r="B51" s="60"/>
-      <c r="C51" s="60"/>
-      <c r="D51" s="60"/>
-      <c r="E51" s="60"/>
+      <c r="B51" s="58"/>
+      <c r="C51" s="58"/>
+      <c r="D51" s="58"/>
+      <c r="E51" s="58"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
@@ -82967,16 +82971,16 @@
       <c r="A53" s="6" t="s">
         <v>725</v>
       </c>
-      <c r="B53" s="61">
+      <c r="B53" s="59">
         <v>84479</v>
       </c>
-      <c r="C53" s="61" t="s">
+      <c r="C53" s="59" t="s">
         <v>726</v>
       </c>
-      <c r="D53" s="61">
+      <c r="D53" s="59">
         <v>9217</v>
       </c>
-      <c r="E53" s="61" t="s">
+      <c r="E53" s="59" t="s">
         <v>684</v>
       </c>
     </row>
@@ -82984,16 +82988,16 @@
       <c r="A54" s="4" t="s">
         <v>727</v>
       </c>
-      <c r="B54" s="62">
+      <c r="B54" s="60">
         <v>62008</v>
       </c>
-      <c r="C54" s="62" t="s">
+      <c r="C54" s="60" t="s">
         <v>728</v>
       </c>
-      <c r="D54" s="62">
+      <c r="D54" s="60">
         <v>6563</v>
       </c>
-      <c r="E54" s="62" t="s">
+      <c r="E54" s="60" t="s">
         <v>696</v>
       </c>
     </row>
@@ -83001,16 +83005,16 @@
       <c r="A55" s="6" t="s">
         <v>729</v>
       </c>
-      <c r="B55" s="61">
+      <c r="B55" s="59">
         <v>37206</v>
       </c>
-      <c r="C55" s="61" t="s">
+      <c r="C55" s="59" t="s">
         <v>730</v>
       </c>
-      <c r="D55" s="61">
+      <c r="D55" s="59">
         <v>3823</v>
       </c>
-      <c r="E55" s="61" t="s">
+      <c r="E55" s="59" t="s">
         <v>691</v>
       </c>
     </row>
@@ -83018,16 +83022,16 @@
       <c r="A56" s="4" t="s">
         <v>731</v>
       </c>
-      <c r="B56" s="62">
+      <c r="B56" s="60">
         <v>35261</v>
       </c>
-      <c r="C56" s="62" t="s">
+      <c r="C56" s="60" t="s">
         <v>732</v>
       </c>
-      <c r="D56" s="62">
+      <c r="D56" s="60">
         <v>3677</v>
       </c>
-      <c r="E56" s="62" t="s">
+      <c r="E56" s="60" t="s">
         <v>658</v>
       </c>
     </row>
@@ -83035,16 +83039,16 @@
       <c r="A57" s="6" t="s">
         <v>733</v>
       </c>
-      <c r="B57" s="61">
+      <c r="B57" s="59">
         <v>23498</v>
       </c>
-      <c r="C57" s="61" t="s">
+      <c r="C57" s="59" t="s">
         <v>734</v>
       </c>
-      <c r="D57" s="61">
+      <c r="D57" s="59">
         <v>2242</v>
       </c>
-      <c r="E57" s="61" t="s">
+      <c r="E57" s="59" t="s">
         <v>719</v>
       </c>
     </row>
@@ -83052,10 +83056,10 @@
       <c r="A60" s="33" t="s">
         <v>735</v>
       </c>
-      <c r="B60" s="60"/>
-      <c r="C60" s="60"/>
-      <c r="D60" s="60"/>
-      <c r="E60" s="60"/>
+      <c r="B60" s="58"/>
+      <c r="C60" s="58"/>
+      <c r="D60" s="58"/>
+      <c r="E60" s="58"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
@@ -83078,16 +83082,16 @@
       <c r="A62" s="4" t="s">
         <v>736</v>
       </c>
-      <c r="B62" s="62">
+      <c r="B62" s="60">
         <v>109701</v>
       </c>
-      <c r="C62" s="62" t="s">
+      <c r="C62" s="60" t="s">
         <v>737</v>
       </c>
-      <c r="D62" s="62">
+      <c r="D62" s="60">
         <v>11377</v>
       </c>
-      <c r="E62" s="62" t="s">
+      <c r="E62" s="60" t="s">
         <v>658</v>
       </c>
     </row>
@@ -83095,16 +83099,16 @@
       <c r="A63" s="6" t="s">
         <v>738</v>
       </c>
-      <c r="B63" s="61">
+      <c r="B63" s="59">
         <v>93841</v>
       </c>
-      <c r="C63" s="61" t="s">
+      <c r="C63" s="59" t="s">
         <v>739</v>
       </c>
-      <c r="D63" s="61">
+      <c r="D63" s="59">
         <v>9164</v>
       </c>
-      <c r="E63" s="61" t="s">
+      <c r="E63" s="59" t="s">
         <v>710</v>
       </c>
     </row>
@@ -83112,16 +83116,16 @@
       <c r="A64" s="4" t="s">
         <v>740</v>
       </c>
-      <c r="B64" s="62">
+      <c r="B64" s="60">
         <v>26711</v>
       </c>
-      <c r="C64" s="62" t="s">
+      <c r="C64" s="60" t="s">
         <v>741</v>
       </c>
-      <c r="D64" s="62">
+      <c r="D64" s="60">
         <v>3389</v>
       </c>
-      <c r="E64" s="62" t="s">
+      <c r="E64" s="60" t="s">
         <v>742</v>
       </c>
     </row>
@@ -83129,16 +83133,16 @@
       <c r="A65" s="6" t="s">
         <v>743</v>
       </c>
-      <c r="B65" s="61">
+      <c r="B65" s="59">
         <v>12199</v>
       </c>
-      <c r="C65" s="61" t="s">
+      <c r="C65" s="59" t="s">
         <v>744</v>
       </c>
-      <c r="D65" s="61">
+      <c r="D65" s="59">
         <v>1592</v>
       </c>
-      <c r="E65" s="61" t="s">
+      <c r="E65" s="59" t="s">
         <v>745</v>
       </c>
     </row>
@@ -83146,10 +83150,10 @@
       <c r="A68" s="33" t="s">
         <v>746</v>
       </c>
-      <c r="B68" s="60"/>
-      <c r="C68" s="60"/>
-      <c r="D68" s="60"/>
-      <c r="E68" s="60"/>
+      <c r="B68" s="58"/>
+      <c r="C68" s="58"/>
+      <c r="D68" s="58"/>
+      <c r="E68" s="58"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
@@ -83170,16 +83174,16 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="4"/>
-      <c r="B70" s="62">
+      <c r="B70" s="60">
         <v>92444</v>
       </c>
-      <c r="C70" s="62" t="s">
+      <c r="C70" s="60" t="s">
         <v>590</v>
       </c>
-      <c r="D70" s="62">
+      <c r="D70" s="60">
         <v>5400</v>
       </c>
-      <c r="E70" s="62" t="s">
+      <c r="E70" s="60" t="s">
         <v>747</v>
       </c>
     </row>
@@ -83187,16 +83191,16 @@
       <c r="A71" s="6" t="s">
         <v>748</v>
       </c>
-      <c r="B71" s="61">
+      <c r="B71" s="59">
         <v>73310</v>
       </c>
-      <c r="C71" s="61" t="s">
+      <c r="C71" s="59" t="s">
         <v>749</v>
       </c>
-      <c r="D71" s="61">
+      <c r="D71" s="59">
         <v>4974</v>
       </c>
-      <c r="E71" s="61" t="s">
+      <c r="E71" s="59" t="s">
         <v>750</v>
       </c>
     </row>
@@ -83204,16 +83208,16 @@
       <c r="A72" s="4" t="s">
         <v>733</v>
       </c>
-      <c r="B72" s="62">
+      <c r="B72" s="60">
         <v>35740</v>
       </c>
-      <c r="C72" s="62" t="s">
+      <c r="C72" s="60" t="s">
         <v>751</v>
       </c>
-      <c r="D72" s="62">
+      <c r="D72" s="60">
         <v>2156</v>
       </c>
-      <c r="E72" s="62" t="s">
+      <c r="E72" s="60" t="s">
         <v>752</v>
       </c>
     </row>
@@ -83221,16 +83225,16 @@
       <c r="A73" s="6" t="s">
         <v>753</v>
       </c>
-      <c r="B73" s="61">
+      <c r="B73" s="59">
         <v>15332</v>
       </c>
-      <c r="C73" s="61" t="s">
+      <c r="C73" s="59" t="s">
         <v>754</v>
       </c>
-      <c r="D73" s="61">
+      <c r="D73" s="59">
         <v>5924</v>
       </c>
-      <c r="E73" s="61" t="s">
+      <c r="E73" s="59" t="s">
         <v>755</v>
       </c>
     </row>
@@ -83238,16 +83242,16 @@
       <c r="A74" s="4" t="s">
         <v>756</v>
       </c>
-      <c r="B74" s="62">
+      <c r="B74" s="60">
         <v>13814</v>
       </c>
-      <c r="C74" s="62" t="s">
+      <c r="C74" s="60" t="s">
         <v>757</v>
       </c>
-      <c r="D74" s="62">
+      <c r="D74" s="60">
         <v>2861</v>
       </c>
-      <c r="E74" s="62" t="s">
+      <c r="E74" s="60" t="s">
         <v>758</v>
       </c>
     </row>
@@ -83255,16 +83259,16 @@
       <c r="A75" s="6" t="s">
         <v>759</v>
       </c>
-      <c r="B75" s="61">
+      <c r="B75" s="59">
         <v>11812</v>
       </c>
-      <c r="C75" s="61" t="s">
+      <c r="C75" s="59" t="s">
         <v>760</v>
       </c>
-      <c r="D75" s="61">
+      <c r="D75" s="59">
         <v>4207</v>
       </c>
-      <c r="E75" s="61" t="s">
+      <c r="E75" s="59" t="s">
         <v>761</v>
       </c>
     </row>
@@ -83272,10 +83276,10 @@
       <c r="A78" s="33" t="s">
         <v>762</v>
       </c>
-      <c r="B78" s="60"/>
-      <c r="C78" s="60"/>
-      <c r="D78" s="60"/>
-      <c r="E78" s="60"/>
+      <c r="B78" s="58"/>
+      <c r="C78" s="58"/>
+      <c r="D78" s="58"/>
+      <c r="E78" s="58"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
@@ -83296,16 +83300,16 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="4"/>
-      <c r="B80" s="62">
+      <c r="B80" s="60">
         <v>92444</v>
       </c>
-      <c r="C80" s="62" t="s">
+      <c r="C80" s="60" t="s">
         <v>590</v>
       </c>
-      <c r="D80" s="62">
+      <c r="D80" s="60">
         <v>5400</v>
       </c>
-      <c r="E80" s="62" t="s">
+      <c r="E80" s="60" t="s">
         <v>747</v>
       </c>
     </row>
@@ -83313,16 +83317,16 @@
       <c r="A81" s="6" t="s">
         <v>694</v>
       </c>
-      <c r="B81" s="61">
+      <c r="B81" s="59">
         <v>78344</v>
       </c>
-      <c r="C81" s="61" t="s">
+      <c r="C81" s="59" t="s">
         <v>763</v>
       </c>
-      <c r="D81" s="61">
+      <c r="D81" s="59">
         <v>5882</v>
       </c>
-      <c r="E81" s="61" t="s">
+      <c r="E81" s="59" t="s">
         <v>764</v>
       </c>
     </row>
@@ -83330,16 +83334,16 @@
       <c r="A82" s="4" t="s">
         <v>692</v>
       </c>
-      <c r="B82" s="62">
+      <c r="B82" s="60">
         <v>35994</v>
       </c>
-      <c r="C82" s="62" t="s">
+      <c r="C82" s="60" t="s">
         <v>765</v>
       </c>
-      <c r="D82" s="62">
+      <c r="D82" s="60">
         <v>11775</v>
       </c>
-      <c r="E82" s="62" t="s">
+      <c r="E82" s="60" t="s">
         <v>766</v>
       </c>
     </row>
@@ -83347,16 +83351,16 @@
       <c r="A83" s="6" t="s">
         <v>689</v>
       </c>
-      <c r="B83" s="61">
+      <c r="B83" s="59">
         <v>35670</v>
       </c>
-      <c r="C83" s="61" t="s">
+      <c r="C83" s="59" t="s">
         <v>767</v>
       </c>
-      <c r="D83" s="61">
+      <c r="D83" s="59">
         <v>2465</v>
       </c>
-      <c r="E83" s="61" t="s">
+      <c r="E83" s="59" t="s">
         <v>768</v>
       </c>
     </row>
@@ -83364,10 +83368,10 @@
       <c r="A86" s="33" t="s">
         <v>769</v>
       </c>
-      <c r="B86" s="60"/>
-      <c r="C86" s="60"/>
-      <c r="D86" s="60"/>
-      <c r="E86" s="60"/>
+      <c r="B86" s="58"/>
+      <c r="C86" s="58"/>
+      <c r="D86" s="58"/>
+      <c r="E86" s="58"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
@@ -83390,16 +83394,16 @@
       <c r="A88" s="4" t="s">
         <v>770</v>
       </c>
-      <c r="B88" s="62">
+      <c r="B88" s="60">
         <v>242452</v>
       </c>
-      <c r="C88" s="62" t="s">
+      <c r="C88" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="D88" s="62">
+      <c r="D88" s="60">
         <v>25522</v>
       </c>
-      <c r="E88" s="62" t="s">
+      <c r="E88" s="60" t="s">
         <v>702</v>
       </c>
     </row>

</xml_diff>